<commit_message>
change name, version, status 0472a83d6e704bb451ec738e0f10c8e1c57d42d9
</commit_message>
<xml_diff>
--- a/ig/mc-add-profiles-dp/StructureDefinition-as-address-extended.xlsx
+++ b/ig/mc-add-profiles-dp/StructureDefinition-as-address-extended.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.0.3</t>
+    <t>0.1.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-05-16T15:52:02+00:00</t>
+    <t>2023-05-16T15:57:02+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>